<commit_message>
complete the qa workflow project prototype and modularize the code for deployment.
</commit_message>
<xml_diff>
--- a/03_live_sessions/01_call_transcript_qa/data/output.xlsx
+++ b/03_live_sessions/01_call_transcript_qa/data/output.xlsx
@@ -454,7 +454,7 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>evaluation_output</t>
+          <t>evaluation_outputs</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
@@ -464,7 +464,7 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>recommendations</t>
+          <t>recommendation</t>
         </is>
       </c>
     </row>
@@ -497,22 +497,22 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>['knowledge_accuracy', 'resolution_quality']</t>
+          <t>["knowledge_accuracy", "resolution_quality"]</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>{'knowledge': {'score': 3, 'reasoning': "The agent acknowledged the customer's issue and indicated they would check the charge, which shows a willingness to assist. However, the transcript does not provide enough information about the agent's knowledge or the accuracy of the information given, as the conversation is incomplete. Therefore, a moderate score is appropriate."}, 'resolution': {'score': 2, 'reasoning': "The agent did not fully resolve the customer's issue as the transcript ends abruptly without confirming the resolution or providing next steps. There is no indication that the agent addressed the double charge or offered a solution."}}</t>
+          <t>{"knowledge": {"knowledge_accuracy_score": 1, "justification": "The agent did not provide any information or resolution to the customer's issue regarding being charged twice for their premium. The response was incomplete and did not address the customer's concern."}, "resolution": {"resolution_quality_score": 2, "issue_resolved": false, "justification": "The agent did not provide a solution or next steps to resolve the customer's issue of being charged twice; they only indicated they would check the issue."}}</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>The agent demonstrated a willingness to assist the customer by acknowledging the issue and indicating they would check the charge. However, the conversation was incomplete, leading to a lack of clarity regarding the agent's knowledge and the resolution of the customer's issue, particularly concerning the double charge.</t>
+          <t>The agent demonstrated a lack of knowledge regarding the customer's issue of being charged twice for their premium service. They failed to provide any relevant information or resolution, resulting in an unresolved issue and inadequate support for the customer.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>['Enhance product knowledge training to ensure agents can provide accurate information and solutions.', 'Implement a structured follow-up process to confirm issue resolution and next steps before ending calls.', "Encourage agents to ask clarifying questions to fully understand the customer's issue and provide comprehensive support.", 'Provide training on handling common issues, such as billing discrepancies, to improve resolution rates.', 'Ensure agents are aware of the importance of completing calls with a clear resolution or action plan.']</t>
+          <t>["Enhance training on common billing issues, particularly double charges, to ensure agents can provide accurate information.", "Implement a standard protocol for addressing customer concerns, including clear next steps for unresolved issues.", "Encourage active listening skills to better understand and address customer concerns during calls.", "Provide agents with access to resources or tools that enable them to quickly find solutions to common problems.", "Conduct regular role-playing exercises to improve response quality and resolution skills in real customer scenarios."]</t>
         </is>
       </c>
     </row>
@@ -545,22 +545,22 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>['knowledge_accuracy', 'resolution_quality']</t>
+          <t>["knowledge_accuracy", "resolution_quality"]</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>{'knowledge': {'score': 2, 'reasoning': "The transcript provides very limited information. The agent acknowledges the customer's concern but does not provide any specific information or resolution regarding the pending claim. This lack of detail makes it difficult to assess the accuracy and clarity of the information provided."}, 'resolution': {'score': 2, 'reasoning': "The agent did not fully resolve the customer's issue regarding the pending claim. There is no indication that the agent provided a solution or next steps for the customer. Additionally, the agent did not confirm resolution before ending the call."}}</t>
+          <t>{"knowledge": {"knowledge_accuracy_score": 2, "justification": "The agent acknowledged the customer's concern but did not provide any specific information regarding the status of the claim or the reasons for the delay, which is crucial for addressing the customer's inquiry."}, "resolution": {"resolution_quality_score": 2, "issue_resolved": false, "justification": "The agent acknowledged the customer's concern but did not provide a clear solution or next steps to resolve the pending claim issue."}}</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>The agent demonstrated a lack of knowledge and resolution skills during the call. They acknowledged the customer's concern but failed to provide specific information or a solution regarding the pending claim, ultimately leaving the customer's issue unresolved.</t>
+          <t>The agent demonstrated a lack of specific knowledge regarding the customer's claim status and failed to provide a resolution or next steps, resulting in an unresolved issue and customer dissatisfaction.</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>['Enhance product knowledge training to ensure agents can provide detailed information about claims and resolutions.', 'Implement a checklist for agents to follow during calls to confirm they have addressed all customer concerns before ending the call.', "Encourage agents to ask clarifying questions to better understand the customer's issue and provide tailored solutions.", 'Provide role-playing scenarios in training sessions to practice handling similar situations effectively.', 'Establish a protocol for agents to follow up with customers if a resolution cannot be provided during the initial call.']</t>
+          <t>["Enhance training on claim processes to ensure agents can provide accurate and detailed information regarding claim statuses.", "Implement a script or guideline for agents to follow when addressing customer inquiries about pending claims, including how to communicate delays effectively.", "Encourage agents to proactively offer next steps or alternative solutions when an issue cannot be resolved immediately.", "Conduct regular role-playing sessions to improve agents' communication skills and their ability to empathize with customers while providing necessary information."]</t>
         </is>
       </c>
     </row>
@@ -593,22 +593,22 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>['tone_empathy', 'resolution_quality']</t>
+          <t>["tone_empathy", "resolution_quality"]</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>{'tone': {'score': 3, 'reasoning': "The agent acknowledged the customer's issue by apologizing for the inconvenience, which is a positive aspect. However, the response lacks further engagement or specific empathy towards the customer's frustration about repeated calls. The tone is polite and professional, but it could be improved by expressing more understanding of the customer's feelings."}, 'resolution': {'score': 2, 'reasoning': "The agent did not fully resolve the customer's issue, as indicated by the customer's frustration and mention of calling multiple times. There is no evidence of clear next steps communicated, and the agent did not confirm resolution before ending the call."}}</t>
+          <t>{"tone": {"tone_empathy_score": 3, "justification": "The agent apologized for the inconvenience, which shows some acknowledgment of the customer's feelings, but the response was brief and lacked further empathy or engagement."}, "resolution": {"resolution_quality_score": 2, "issue_resolved": false, "justification": "The agent apologized for the inconvenience but did not provide a clear solution or steps to resolve the customer's ongoing issue."}}</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>The agent demonstrated a polite and professional tone, acknowledging the customer's issue with an apology. However, the interaction fell short in terms of empathy and resolution, as the customer's ongoing frustration was not adequately addressed, and no clear next steps were communicated.</t>
+          <t>The agent demonstrated a basic level of empathy by apologizing for the customer's inconvenience but failed to engage further or provide a clear resolution to the issue, resulting in an unresolved customer concern.</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>["Enhance empathy by acknowledging the customer's feelings more explicitly, especially regarding their frustration from repeated calls.", 'Ensure that all customer issues are fully resolved during the call by actively confirming resolution before ending the conversation.', 'Communicate clear next steps to the customer, outlining what actions will be taken to address their issue and when they can expect follow-up.', "Engage in active listening to better understand the customer's concerns and provide tailored responses based on their specific situation."]</t>
+          <t>["Enhance empathetic communication by actively listening to the customer and acknowledging their feelings more deeply.", "Provide clear and actionable solutions to the customer's issues, ensuring they understand the steps being taken.", "Follow up with the customer to confirm resolution and satisfaction, reinforcing a commitment to service.", "Engage in role-playing scenarios to practice handling difficult calls and improving resolution strategies."]</t>
         </is>
       </c>
     </row>
@@ -637,26 +637,26 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0.9</v>
+        <v>0.95</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>['knowledge_accuracy']</t>
+          <t>["knowledge_accuracy"]</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>{'knowledge': {'score': 3, 'reasoning': "The transcript does not provide enough information about the agent's explanation of the coverage details. While the agent indicates they will explain, there is no actual content to evaluate for accuracy or clarity. Therefore, a moderate score is appropriate."}}</t>
+          <t>{"knowledge": {"knowledge_accuracy_score": 3, "justification": "The agent's response indicates willingness to explain coverage details, but the lack of specific information in the provided transcript makes it unclear whether the agent accurately addressed the customer's question."}}</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>The agent demonstrated a willingness to explain coverage details but failed to provide any actual content during the call, resulting in a lack of clarity and understanding for the customer.</t>
+          <t>The agent demonstrated a willingness to explain coverage details, but the lack of specific information in the response left the customer's question inadequately addressed. This indicates a need for improvement in knowledge application and clarity in communication.</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>['Ensure that the agent provides clear and detailed explanations of coverage details during calls.', 'Conduct training sessions focused on effective communication and clarity in explanations.', 'Implement a checklist for agents to follow when discussing coverage to ensure all necessary information is covered.', 'Encourage role-playing exercises to practice delivering information in a concise and understandable manner.', 'Review and analyze successful calls to identify best practices for explaining complex topics.']</t>
+          <t>["Enhance product knowledge training to ensure agents can provide specific and accurate information regarding coverage details.", "Implement role-playing scenarios to practice responding to common customer inquiries with clarity and confidence.", "Encourage agents to ask clarifying questions to fully understand customer concerns before providing information.", "Develop a resource guide that agents can reference during calls to quickly access detailed coverage information.", "Conduct regular feedback sessions to review call transcripts and identify areas for improvement in knowledge application."]</t>
         </is>
       </c>
     </row>

</xml_diff>